<commit_message>
refactor(web-dashboard): remove Istimara permit radar card and sync import templates
</commit_message>
<xml_diff>
--- a/frontend/web-dashboard/public/templates/MERCON_Drivers_Import_Template.xlsx
+++ b/frontend/web-dashboard/public/templates/MERCON_Drivers_Import_Template.xlsx
@@ -608,7 +608,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="85" customWidth="1" min="2" max="2"/>
@@ -760,7 +760,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>

</xml_diff>